<commit_message>
Lowercase the sample rider codes; read benefit rules in long-form
- Lowercase the sample rider codes (dth_main, adb, hosp, cancer, ann,
  mat) across the bundled sample, the examples data and the tutorial, so
  the wide columns read as clean snake_case -- cancer_benefit, not
  CANCER_benefit.
- The long-form coverages reader now picks up optional waiting,
  reduction_end and reduction_factor columns, so a coverage's waiting
  and reduced-benefit periods can be set from the file.
</commit_message>
<xml_diff>
--- a/examples/data/assumptions.xlsx
+++ b/examples/data/assumptions.xlsx
@@ -2405,7 +2405,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DTH_MAIN</t>
+          <t>dth_main</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANN</t>
+          <t>ann</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>mat</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2568,7 +2568,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2584,7 +2584,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2600,7 +2600,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2616,7 +2616,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2632,7 +2632,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2648,7 +2648,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2664,7 +2664,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2680,7 +2680,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2696,7 +2696,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2712,7 +2712,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2728,7 +2728,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2744,7 +2744,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2760,7 +2760,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2776,7 +2776,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2792,7 +2792,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2808,7 +2808,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2824,7 +2824,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2840,7 +2840,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2856,7 +2856,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2872,7 +2872,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2888,7 +2888,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2904,7 +2904,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2920,7 +2920,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2936,7 +2936,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2952,7 +2952,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2968,7 +2968,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2984,7 +2984,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3000,7 +3000,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3016,7 +3016,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3032,7 +3032,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3048,7 +3048,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -3064,7 +3064,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -3080,7 +3080,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -3096,7 +3096,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -3112,7 +3112,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -3128,7 +3128,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3144,7 +3144,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3160,7 +3160,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3176,7 +3176,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3192,7 +3192,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3208,7 +3208,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3224,7 +3224,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3240,7 +3240,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3256,7 +3256,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -3272,7 +3272,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3288,7 +3288,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -3304,7 +3304,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -3320,7 +3320,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -3336,7 +3336,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -3352,7 +3352,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -3368,7 +3368,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -3384,7 +3384,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -3400,7 +3400,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -3416,7 +3416,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -3432,7 +3432,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -3448,7 +3448,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -3464,7 +3464,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -3480,7 +3480,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3496,7 +3496,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -3512,7 +3512,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -3528,7 +3528,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -3544,7 +3544,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -3560,7 +3560,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -3576,7 +3576,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3592,7 +3592,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -3608,7 +3608,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -3624,7 +3624,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -3640,7 +3640,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -3656,7 +3656,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -3672,7 +3672,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -3688,7 +3688,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -3704,7 +3704,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -3720,7 +3720,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -3736,7 +3736,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -3752,7 +3752,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -3768,7 +3768,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -3784,7 +3784,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -3800,7 +3800,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -3816,7 +3816,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -3832,7 +3832,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -3848,7 +3848,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -3864,7 +3864,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -3880,7 +3880,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -3896,7 +3896,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -3912,7 +3912,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -3928,7 +3928,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -3944,7 +3944,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -3960,7 +3960,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -3976,7 +3976,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -3992,7 +3992,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -4008,7 +4008,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -4024,7 +4024,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -4040,7 +4040,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -4056,7 +4056,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -4072,7 +4072,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -4088,7 +4088,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -4104,7 +4104,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -4120,7 +4120,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -4136,7 +4136,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -4152,7 +4152,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -4168,7 +4168,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -4184,7 +4184,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -4200,7 +4200,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -4216,7 +4216,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -4232,7 +4232,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -4248,7 +4248,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -4264,7 +4264,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -4280,7 +4280,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -4296,7 +4296,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -4312,7 +4312,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -4328,7 +4328,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -4344,7 +4344,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -4360,7 +4360,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -4376,7 +4376,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -4392,7 +4392,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -4408,7 +4408,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -4424,7 +4424,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -4440,7 +4440,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -4456,7 +4456,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -4472,7 +4472,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -4488,7 +4488,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -4504,7 +4504,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -4520,7 +4520,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -4536,7 +4536,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -4552,7 +4552,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -4568,7 +4568,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -4584,7 +4584,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -4600,7 +4600,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -4616,7 +4616,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -4632,7 +4632,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -4648,7 +4648,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -4664,7 +4664,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -4680,7 +4680,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -4696,7 +4696,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -4712,7 +4712,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -4728,7 +4728,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -4744,7 +4744,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -4760,7 +4760,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -4776,7 +4776,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -4792,7 +4792,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -4808,7 +4808,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -4824,7 +4824,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>adb</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -4840,7 +4840,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -4856,7 +4856,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -4872,7 +4872,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -4888,7 +4888,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -4904,7 +4904,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -4920,7 +4920,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -4936,7 +4936,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -4952,7 +4952,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -4968,7 +4968,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -4984,7 +4984,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -5000,7 +5000,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -5016,7 +5016,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -5032,7 +5032,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -5048,7 +5048,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -5064,7 +5064,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -5080,7 +5080,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -5096,7 +5096,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -5112,7 +5112,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -5128,7 +5128,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -5144,7 +5144,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -5160,7 +5160,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -5176,7 +5176,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -5192,7 +5192,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -5208,7 +5208,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -5224,7 +5224,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -5240,7 +5240,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -5256,7 +5256,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -5272,7 +5272,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -5288,7 +5288,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -5304,7 +5304,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -5320,7 +5320,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -5336,7 +5336,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -5352,7 +5352,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -5368,7 +5368,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -5384,7 +5384,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -5400,7 +5400,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -5416,7 +5416,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -5432,7 +5432,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -5448,7 +5448,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -5464,7 +5464,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -5480,7 +5480,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -5496,7 +5496,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -5512,7 +5512,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -5528,7 +5528,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -5544,7 +5544,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -5560,7 +5560,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -5576,7 +5576,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -5592,7 +5592,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -5608,7 +5608,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -5624,7 +5624,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -5640,7 +5640,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -5656,7 +5656,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -5672,7 +5672,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -5688,7 +5688,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -5704,7 +5704,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -5720,7 +5720,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -5736,7 +5736,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -5752,7 +5752,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -5768,7 +5768,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -5784,7 +5784,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -5800,7 +5800,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -5816,7 +5816,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -5832,7 +5832,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -5848,7 +5848,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -5864,7 +5864,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -5880,7 +5880,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -5896,7 +5896,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -5912,7 +5912,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -5928,7 +5928,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -5944,7 +5944,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -5960,7 +5960,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -5976,7 +5976,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -5992,7 +5992,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -6008,7 +6008,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -6024,7 +6024,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -6040,7 +6040,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -6056,7 +6056,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -6072,7 +6072,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -6088,7 +6088,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -6104,7 +6104,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -6120,7 +6120,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -6136,7 +6136,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -6152,7 +6152,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -6168,7 +6168,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -6184,7 +6184,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -6200,7 +6200,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -6216,7 +6216,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -6232,7 +6232,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -6248,7 +6248,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -6264,7 +6264,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -6280,7 +6280,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -6296,7 +6296,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -6312,7 +6312,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -6328,7 +6328,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -6344,7 +6344,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -6360,7 +6360,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -6376,7 +6376,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -6392,7 +6392,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -6408,7 +6408,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -6424,7 +6424,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -6440,7 +6440,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -6456,7 +6456,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -6472,7 +6472,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -6488,7 +6488,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -6504,7 +6504,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -6520,7 +6520,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -6536,7 +6536,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -6552,7 +6552,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -6568,7 +6568,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -6584,7 +6584,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -6600,7 +6600,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -6616,7 +6616,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -6632,7 +6632,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -6648,7 +6648,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -6664,7 +6664,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -6680,7 +6680,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -6696,7 +6696,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -6712,7 +6712,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -6728,7 +6728,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -6744,7 +6744,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -6760,7 +6760,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -6776,7 +6776,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -6792,7 +6792,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -6808,7 +6808,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -6824,7 +6824,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -6840,7 +6840,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -6856,7 +6856,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -6872,7 +6872,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -6888,7 +6888,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -6904,7 +6904,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -6920,7 +6920,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -6936,7 +6936,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -6952,7 +6952,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -6968,7 +6968,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -6984,7 +6984,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -7000,7 +7000,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -7016,7 +7016,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -7032,7 +7032,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -7048,7 +7048,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -7064,7 +7064,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -7080,7 +7080,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -7096,7 +7096,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>hosp</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -7112,7 +7112,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -7128,7 +7128,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -7144,7 +7144,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -7160,7 +7160,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -7176,7 +7176,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -7192,7 +7192,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -7208,7 +7208,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -7224,7 +7224,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -7240,7 +7240,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -7256,7 +7256,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -7272,7 +7272,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -7288,7 +7288,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -7304,7 +7304,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -7320,7 +7320,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -7336,7 +7336,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -7352,7 +7352,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -7368,7 +7368,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -7384,7 +7384,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -7400,7 +7400,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -7416,7 +7416,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -7432,7 +7432,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -7448,7 +7448,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -7464,7 +7464,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -7480,7 +7480,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -7496,7 +7496,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -7512,7 +7512,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -7528,7 +7528,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -7544,7 +7544,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -7560,7 +7560,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -7576,7 +7576,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -7592,7 +7592,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -7608,7 +7608,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -7624,7 +7624,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -7640,7 +7640,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -7656,7 +7656,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -7672,7 +7672,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -7688,7 +7688,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -7704,7 +7704,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -7720,7 +7720,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -7736,7 +7736,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -7752,7 +7752,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B326" t="n">
@@ -7768,7 +7768,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B327" t="n">
@@ -7784,7 +7784,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B328" t="n">
@@ -7800,7 +7800,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B329" t="n">
@@ -7816,7 +7816,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B330" t="n">
@@ -7832,7 +7832,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B331" t="n">
@@ -7848,7 +7848,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B332" t="n">
@@ -7864,7 +7864,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B333" t="n">
@@ -7880,7 +7880,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B334" t="n">
@@ -7896,7 +7896,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B335" t="n">
@@ -7912,7 +7912,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B336" t="n">
@@ -7928,7 +7928,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B337" t="n">
@@ -7944,7 +7944,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B338" t="n">
@@ -7960,7 +7960,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B339" t="n">
@@ -7976,7 +7976,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B340" t="n">
@@ -7992,7 +7992,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B341" t="n">
@@ -8008,7 +8008,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B342" t="n">
@@ -8024,7 +8024,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B343" t="n">
@@ -8040,7 +8040,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B344" t="n">
@@ -8056,7 +8056,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B345" t="n">
@@ -8072,7 +8072,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B346" t="n">
@@ -8088,7 +8088,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B347" t="n">
@@ -8104,7 +8104,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B348" t="n">
@@ -8120,7 +8120,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B349" t="n">
@@ -8136,7 +8136,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B350" t="n">
@@ -8152,7 +8152,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B351" t="n">
@@ -8168,7 +8168,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B352" t="n">
@@ -8184,7 +8184,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B353" t="n">
@@ -8200,7 +8200,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B354" t="n">
@@ -8216,7 +8216,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B355" t="n">
@@ -8232,7 +8232,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B356" t="n">
@@ -8248,7 +8248,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B357" t="n">
@@ -8264,7 +8264,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B358" t="n">
@@ -8280,7 +8280,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B359" t="n">
@@ -8296,7 +8296,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B360" t="n">
@@ -8312,7 +8312,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B361" t="n">
@@ -8328,7 +8328,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B362" t="n">
@@ -8344,7 +8344,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B363" t="n">
@@ -8360,7 +8360,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B364" t="n">
@@ -8376,7 +8376,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B365" t="n">
@@ -8392,7 +8392,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B366" t="n">
@@ -8408,7 +8408,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B367" t="n">
@@ -8424,7 +8424,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B368" t="n">
@@ -8440,7 +8440,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B369" t="n">
@@ -8456,7 +8456,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B370" t="n">
@@ -8472,7 +8472,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B371" t="n">
@@ -8488,7 +8488,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B372" t="n">
@@ -8504,7 +8504,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B373" t="n">
@@ -8520,7 +8520,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B374" t="n">
@@ -8536,7 +8536,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B375" t="n">
@@ -8552,7 +8552,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B376" t="n">
@@ -8568,7 +8568,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B377" t="n">
@@ -8584,7 +8584,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B378" t="n">
@@ -8600,7 +8600,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B379" t="n">
@@ -8616,7 +8616,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B380" t="n">
@@ -8632,7 +8632,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B381" t="n">
@@ -8648,7 +8648,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B382" t="n">
@@ -8664,7 +8664,7 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B383" t="n">
@@ -8680,7 +8680,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B384" t="n">
@@ -8696,7 +8696,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B385" t="n">
@@ -8712,7 +8712,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B386" t="n">
@@ -8728,7 +8728,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B387" t="n">
@@ -8744,7 +8744,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B388" t="n">
@@ -8760,7 +8760,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B389" t="n">
@@ -8776,7 +8776,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B390" t="n">
@@ -8792,7 +8792,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B391" t="n">
@@ -8808,7 +8808,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B392" t="n">
@@ -8824,7 +8824,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B393" t="n">
@@ -8840,7 +8840,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B394" t="n">
@@ -8856,7 +8856,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B395" t="n">
@@ -8872,7 +8872,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B396" t="n">
@@ -8888,7 +8888,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B397" t="n">
@@ -8904,7 +8904,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B398" t="n">
@@ -8920,7 +8920,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B399" t="n">
@@ -8936,7 +8936,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B400" t="n">
@@ -8952,7 +8952,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B401" t="n">
@@ -8968,7 +8968,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B402" t="n">
@@ -8984,7 +8984,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B403" t="n">
@@ -9000,7 +9000,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B404" t="n">
@@ -9016,7 +9016,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B405" t="n">
@@ -9032,7 +9032,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B406" t="n">
@@ -9048,7 +9048,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B407" t="n">
@@ -9064,7 +9064,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B408" t="n">
@@ -9080,7 +9080,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B409" t="n">
@@ -9096,7 +9096,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B410" t="n">
@@ -9112,7 +9112,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B411" t="n">
@@ -9128,7 +9128,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B412" t="n">
@@ -9144,7 +9144,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B413" t="n">
@@ -9160,7 +9160,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B414" t="n">
@@ -9176,7 +9176,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B415" t="n">
@@ -9192,7 +9192,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B416" t="n">
@@ -9208,7 +9208,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B417" t="n">
@@ -9224,7 +9224,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B418" t="n">
@@ -9240,7 +9240,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B419" t="n">
@@ -9256,7 +9256,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B420" t="n">
@@ -9272,7 +9272,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B421" t="n">
@@ -9288,7 +9288,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B422" t="n">
@@ -9304,7 +9304,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B423" t="n">
@@ -9320,7 +9320,7 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B424" t="n">
@@ -9336,7 +9336,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B425" t="n">
@@ -9352,7 +9352,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B426" t="n">
@@ -9368,7 +9368,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>cancer</t>
         </is>
       </c>
       <c r="B427" t="n">

</xml_diff>

<commit_message>
refactor!: rename product / channel to product_code / channel_code
Bring segment routing keys in line with the rest of the codebase, where
every cross-file join key already carries a ``_code`` suffix
(``coverage_code``, ``table_id``, ...). The (product, channel) tuple
itself stays the segment routing key -- only the column and field names
change.

- ``ModelPoints.product`` / ``.channel`` → ``.product_code`` / ``.channel_code``
- Assumptions workbook ``segments`` and ``ae_factors`` sheets:
  ``product`` / ``channel`` column headers → ``product_code`` /
  ``channel_code``
- Sample policies CSV header renamed in lockstep
- All engine / trace / io / test references updated; the dict basis is
  still keyed by the raw string tuple
</commit_message>
<xml_diff>
--- a/examples/data/assumptions.xlsx
+++ b/examples/data/assumptions.xlsx
@@ -429,12 +429,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>product_code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>channel_code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -28158,12 +28158,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>product_code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>channel_code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">

</xml_diff>